<commit_message>
Add suggested replies to every fresh lead and move the reply column forward
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015dXgfxu1ugCxsD9bCGxkqs
</commit_message>
<xml_diff>
--- a/lynkk-reddit-leads/results/2026-10-27/fresh_keyword_leads.xlsx
+++ b/lynkk-reddit-leads/results/2026-10-27/fresh_keyword_leads.xlsx
@@ -427,16 +427,16 @@
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="80" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="45" customWidth="1" min="13" max="13"/>
-    <col width="80" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
     <col width="16" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
     <col width="35" customWidth="1" min="17" max="17"/>
@@ -461,57 +461,57 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>suggested_reply</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>pain_point</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>profile_link</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>type</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>thread_link</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>keyword_matched</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>posted</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>relevance_score</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>intent</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>pain_point</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>suggested_reply</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
@@ -553,55 +553,55 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>post</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/PLAUDAI/comments/1x1tha4/lawyers_using_plaud_or_other_ai_notetakers_for/</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>On the in-person side, a laptop's built-in mic is usually fine for two or three people across a desk, but a cheap USB boundary mic in the middle of the table makes a bigger difference to transcript accuracy than switching apps. For your weeks-later problem, judge tools on what the summary keeps: decisions, open questions and action items, with timestamps that jump back to the recording so you can check the exact wording before drafting. For a fair test, run the same real consultation through two or three tools and compare them side by side. On confidentiality, ask each vendor in writing whether they train on your recordings, where data is stored and how deletion works, and get client consent on the record at the start.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Lawyers using Plaud or other AI note-takers for client consultations — what has your experience been?</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Loses important details from client consultations because weeks pass between the meeting and drafting, and handwritten notes miss context.</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
           <t>https://www.reddit.com/user/Party_History2839/</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>post</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>https://www.reddit.com/r/PLAUDAI/comments/1x1tha4/lawyers_using_plaud_or_other_ai_notetakers_for/</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/PLAUDAI/comments/1x1tha4/lawyers_using_plaud_or_other_ai_notetakers_for/</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Lawyers using Plaud or other AI note-takers for client consultations — what has your experience been?</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>"Otter" alternative</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="K2" s="2" t="n">
+      <c r="M2" s="2" t="n">
         <v>82</v>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>comparison</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>Loses important details from client consultations because weeks pass between the meeting and drafting, and handwritten notes miss context.</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>On the in-person side, a laptop's built-in mic is usually fine for two or three people across a desk, but a cheap USB boundary mic in the middle of the table makes a bigger difference to transcript accuracy than switching apps. For your weeks-later problem, judge tools on what the summary keeps: decisions, open questions and action items, with timestamps that jump back to the recording so you can check the exact wording before drafting. For a fair test, run the same real consultation through two or three tools and compare them side by side. On confidentiality, ask each vendor in writing whether they train on your recordings, where data is stored and how deletion works, and get client consent on the record at the start.</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -643,56 +643,56 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/user/Prior_Conference_257/</t>
+          <t>post</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>post</t>
+          <t>https://www.reddit.com/r/projectmanagers/comments/1xcjt5q/best_ai_meeting_notetaker_that_works_across_teams/</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/projectmanagers/comments/1xcjt5q/best_ai_meeting_notetaker_that_works_across_teams/</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/projectmanagers/comments/1xcjt5q/best_ai_meeting_notetaker_that_works_across_teams/</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Best AI meeting notetaker that works across Teams / Zoom / Google Meet</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>"note taker" sales</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="n">
-        <v>80</v>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>tool_recommendation</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>Ops lead must pick one AI note taker that works on Teams, Zoom and Meet, with admin controls, to replace random free tools.</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>For mixed platforms the first decision is bot or no bot. A bot that joins Meet, Zoom and Teams links works the same everywhere but shows up as a participant, which some clients push back on. A desktop or browser recorder stays out of the call but needs each person to install it. For admin controls, ask every vendor how notes are shared by default, whether people can keep a note personal, and whether they train on your recordings.
 Lynkk is one to put on the shortlist next to Otter, Fireflies and Granola. It has a meeting bot for Meet, Zoom and Teams plus a no-bot Mac app and Chrome extension, and a company workspace where admins can read workspace notes (every admin read is logged) while people can mark notes personal. Two limits to check: workspaces cap at 10 seats, and the desktop app is Mac only.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Best AI meeting notetaker that works across Teams / Zoom / Google Meet</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Ops lead must pick one AI note taker that works on Teams, Zoom and Meet, with admin controls, to replace random free tools.</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/user/Prior_Conference_257/</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/projectmanagers/comments/1xcjt5q/best_ai_meeting_notetaker_that_works_across_teams/</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>"note taker" sales</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>tool_recommendation</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
@@ -734,56 +734,56 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/user/AgreeableEffect717/</t>
+          <t>post</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>post</t>
+          <t>https://www.reddit.com/r/RecruitmentAgencies/comments/1x4s9f8/just_lost_a_candidate_because_two_of_us/</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/RecruitmentAgencies/comments/1x4s9f8/just_lost_a_candidate_because_two_of_us/</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/RecruitmentAgencies/comments/1x4s9f8/just_lost_a_candidate_because_two_of_us/</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Just lost a candidate because two of us remembered the same interview completely differently</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>"note taker" sales</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>tool_recommendation</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>Two interviewers remembered a candidate's answers differently, no usable notes, lost the candidate; wants an AI note taker for interviews.</t>
-        </is>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>For interviews, say at the start that the call is recorded for notes and give the candidate a real option to say no. Most people are fine once it's explained. Then run the debrief against the recording instead of memory, which is exactly the "team of five" problem. A short scorecard also helps: scope of past roles, examples given, concerns, what to probe next round.
 Lynkk is worth testing for this alongside Otter or Fireflies. Its free brief lists key takeaways with timestamps that play the recording from that moment, so you can check what was actually said in seconds, and you can share the note with the other interviewer by email. In-person interviews work from the browser; there's no phone app.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Just lost a candidate because two of us remembered the same interview completely differently</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Two interviewers remembered a candidate's answers differently, no usable notes, lost the candidate; wants an AI note taker for interviews.</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/user/AgreeableEffect717/</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/RecruitmentAgencies/comments/1x4s9f8/just_lost_a_candidate_because_two_of_us/</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>"note taker" sales</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>tool_recommendation</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
@@ -825,56 +825,56 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/user/No_Lawyer6832/</t>
+          <t>post</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>post</t>
+          <t>https://www.reddit.com/r/CRMSoftware/comments/1vkn5m7/our_sales_calls_are_a_black_hole_nobody_takes/</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/CRMSoftware/comments/1vkn5m7/our_sales_calls_are_a_black_hole_nobody_takes/</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/CRMSoftware/comments/1vkn5m7/our_sales_calls_are_a_black_hole_nobody_takes/</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Our sales calls are a black hole. Nobody takes good notes and follow ups are inconsistent. How do you fix this?</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>"note taker" sales</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="n">
-        <v>76</v>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>problem_seeking_solution</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>Sales call notes are vague or missing, so follow-ups and CS handoffs lose context.</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>Templates rarely fix this because the problem is that notes depend on memory after the call. Record the calls instead, and make the summary the handoff document: decisions, next steps with owners and dates, and open questions, with a link back to the moment in the recording when CS needs the exact wording. Then the only manual step is pasting the next steps into the CRM.
 For a team of 8, Lynkk is worth a look alongside Gong or Fireflies: it records calls without a bot, writes that kind of brief after every call, and on the paid plan you can ask questions across all your calls with a customer. It doesn't sync to the CRM, so that step stays manual.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Our sales calls are a black hole. Nobody takes good notes and follow ups are inconsistent. How do you fix this?</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Sales call notes are vague or missing, so follow-ups and CS handoffs lose context.</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/user/No_Lawyer6832/</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/CRMSoftware/comments/1vkn5m7/our_sales_calls_are_a_black_hole_nobody_takes/</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>"note taker" sales</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>problem_seeking_solution</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
@@ -916,56 +916,56 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/user/pedrogalopp/</t>
+          <t>post</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>post</t>
+          <t>https://www.reddit.com/r/techsales/comments/1xboww3/ai_call_summaries_too_generic_for_sales/</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/techsales/comments/1xboww3/ai_call_summaries_too_generic_for_sales/</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/techsales/comments/1xboww3/ai_call_summaries_too_generic_for_sales/</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>AI call summaries too generic for sales？</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>"note taker" sales</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="n">
-        <v>74</v>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>tool_recommendation</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>AI call summaries miss the small sales details, so they still dig through transcripts.</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>Generic summaries usually come from a general meeting template. The fix is a sales-specific structure: pain points in the customer's words, budget and timeline, objections, who else is involved, and next steps with dates. And for the small details, being able to click a line and hear that moment beats rereading the transcript.
 Worth trying Lynkk next to Gong, Fathom or Fireflies: it has a dedicated Sales Call summary format, every takeaway links back to the moment in the recording, and you can ask questions across all your calls with a customer. The sales format is on the paid plan; the basic brief is free.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>AI call summaries too generic for sales？</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>AI call summaries miss the small sales details, so they still dig through transcripts.</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/user/pedrogalopp/</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/techsales/comments/1xboww3/ai_call_summaries_too_generic_for_sales/</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>"note taker" sales</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>tool_recommendation</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
@@ -1007,56 +1007,56 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/user/jnjsch/</t>
+          <t>post</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>post</t>
+          <t>https://www.reddit.com/r/ObsidianMD/comments/1vpg175/best_workflow_for_recording_inpersononline/</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/ObsidianMD/comments/1vpg175/best_workflow_for_recording_inpersononline/</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/ObsidianMD/comments/1vpg175/best_workflow_for_recording_inpersononline/</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Best workflow for recording in-person/online meetings and syncing transcripts + AI notes into Obsidian? (Granola alternative)</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>Granola alternative</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-15</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>comparison</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>Their Granola plus Obsidian sync setup broke after Granola locked down API access, so they need a new way to capture meetings into their vault.</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>Since the sync part is what broke, I'd pick capture and Obsidian export separately. For capture, anything that records your mic and system audio without a bot covers online calls, and a laptop mic is fine for in-person. For the vault, the most durable setup is a tool that gives you plain text or Markdown you can paste or drop into a folder, so a plugin breaking can't strand your notes again.
 Lynkk is one to look at for the capture side: no-bot recording for calls, in-person from the browser, and summaries with decisions and action items. Check how you'd get notes into the vault before committing, since there's no Obsidian plugin.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Best workflow for recording in-person/online meetings and syncing transcripts + AI notes into Obsidian? (Granola alternative)</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Their Granola plus Obsidian sync setup broke after Granola locked down API access, so they need a new way to capture meetings into their vault.</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/user/jnjsch/</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/ObsidianMD/comments/1vpg175/best_workflow_for_recording_inpersononline/</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Granola alternative</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>comparison</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
@@ -1098,56 +1098,56 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/user/newtothis30394/</t>
+          <t>post</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>post</t>
+          <t>https://www.reddit.com/r/Journalism/comments/1wzm13h/newsroom_is_canceling_otter/</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/Journalism/comments/1wzm13h/newsroom_is_canceling_otter/</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/Journalism/comments/1wzm13h/newsroom_is_canceling_otter/</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Newsroom is canceling Otter</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>"Otter" alternative</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>comparison</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>Newsroom is cancelling Otter; needs live transcription and audio/text sync for reporting.</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>For reporting, the two things to test are live transcription and clicking any line to play the audio from that point, since that's what saves time checking quotes. Also check language support if you interview in more than one language, and ask whether the tool trains on your recordings, which matters for sources.
 Worth comparing Lynkk with Fireflies, Descript or Rev. Lynkk shows live words while it records (Mac app or meeting bot), every takeaway in the note plays the recording from that moment, it transcribes 17 languages, and it never trains on your conversations. One limit: no phone app, so in-person interviews mean recording from a laptop.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Newsroom is canceling Otter</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Newsroom is cancelling Otter; needs live transcription and audio/text sync for reporting.</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/user/newtothis30394/</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/Journalism/comments/1wzm13h/newsroom_is_canceling_otter/</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>"Otter" alternative</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>comparison</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
@@ -1189,56 +1189,56 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/user/Big-Personality-9618/</t>
+          <t>post</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>post</t>
+          <t>https://www.reddit.com/r/Entrepreneurs/comments/1wsbiws/otter_alternative_for_business_when_everyone_has/</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/Entrepreneurs/comments/1wsbiws/otter_alternative_for_business_when_everyone_has/</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/Entrepreneurs/comments/1wsbiws/otter_alternative_for_business_when_everyone_has/</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>Otter alternative for business when everyone has a separate account?</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>Otter alternative</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>comparison</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>Individual Otter accounts mean retention varies, visibility is limited and offboarding means chasing accounts.</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>On the migration worry: plan to export each person's Otter history to files before switching and store it centrally, rather than expecting a new tool to import it. Most don't do that cleanly, and it means the old history isn't hostage to whichever tool you choose. Then switch new meetings only, so people aren't asked to change everything at once.
 For the management side on small teams, Lynkk's workspaces cover what you listed: colleagues join by company email domain, admins can read workspace-visible notes with every admin read logged, and people can still mark a note personal. They cap at 10 seats, so it fits small clients only.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Otter alternative for business when everyone has a separate account?</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Individual Otter accounts mean retention varies, visibility is limited and offboarding means chasing accounts.</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/user/Big-Personality-9618/</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/Entrepreneurs/comments/1wsbiws/otter_alternative_for_business_when_everyone_has/</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Otter alternative</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>comparison</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
@@ -1280,56 +1280,56 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/user/This_Yogurtcloset930/</t>
+          <t>post</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>post</t>
+          <t>https://www.reddit.com/r/sales/comments/1vyh8ld/ai_note_taker_adhd/</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/sales/comments/1vyh8ld/ai_note_taker_adhd/</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/sales/comments/1vyh8ld/ai_note_taker_adhd/</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>AI note taker ADHD</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>"note taker" sales</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="n">
-        <v>66</v>
-      </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>high_purchase_intent</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>Recaps arrive too late to send the follow-up while the call is fresh.</t>
-        </is>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>The delay is often the org's setup rather than the tool, so ask your admin whether recaps can go to you directly instead of through an approval or sync step. Either way, a habit that helps with ADHD: before you hang up, say the next steps out loud and type three bullets into the follow-up email draft right away, then let the recap fill in the details.
 If you want a separate free option, Lynkk is one to test alongside Fathom or Otter: it records Zoom, Meet and Teams without a bot and emails you the summary after each meeting.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>AI note taker ADHD</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Recaps arrive too late to send the follow-up while the call is fresh.</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/user/This_Yogurtcloset930/</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/sales/comments/1vyh8ld/ai_note_taker_adhd/</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>"note taker" sales</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>high_purchase_intent</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
@@ -1371,56 +1371,56 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/user/Morphius007/</t>
+          <t>post</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>post</t>
+          <t>https://www.reddit.com/r/MyAIAssistant/comments/1w82fkm/my_ai_summarized_the_meeting_it_dropped_the_only/</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/MyAIAssistant/comments/1w82fkm/my_ai_summarized_the_meeting_it_dropped_the_only/</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/MyAIAssistant/comments/1w82fkm/my_ai_summarized_the_meeting_it_dropped_the_only/</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>My AI summarized the meeting. It dropped the only decision that needed an owner.</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>"meeting assistant" AI</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-05</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="n">
-        <v>66</v>
-      </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>general_discussion</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>Summary dropped the one decision that needed an owner; asks what people require from meeting assistants.</t>
-        </is>
-      </c>
-      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>Same list here, plus one: every action item should link back to the moment it was said, so you can check the exact wording before acting on it, especially for money or customer promises. And decisions should be their own section, not something you dig out of prose.
 Lynkk does this in its free brief: decisions with context, action items with owner, due date and priority, open questions, all timestamped. Fireflies and Otter are the other common ones to compare. Anything touching payments still deserves a human check before it goes out.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>My AI summarized the meeting. It dropped the only decision that needed an owner.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Summary dropped the one decision that needed an owner; asks what people require from meeting assistants.</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/user/Morphius007/</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/MyAIAssistant/comments/1w82fkm/my_ai_summarized_the_meeting_it_dropped_the_only/</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>"meeting assistant" AI</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>general_discussion</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
@@ -1462,56 +1462,56 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/user/Sash19/</t>
+          <t>post</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>post</t>
+          <t>https://www.reddit.com/r/AI_Agents/comments/1wq1vrs/any_fathom_ai_alternatives_that_work_better_with/</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/AI_Agents/comments/1wq1vrs/any_fathom_ai_alternatives_that_work_better_with/</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/AI_Agents/comments/1wq1vrs/any_fathom_ai_alternatives_that_work_better_with/</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>Any Fathom AI alternatives that work better with agent workflows?</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>"Fathom" alternative</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="n">
-        <v>66</v>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>comparison</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>Getting enough context from past meetings for follow-ups, tasks and older decisions means moving transcripts around by hand.</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>Two setups seem to work. One is piping transcripts into your agent through an integration like the MCP route you're testing, which is flexible but means your agent does the retrieval work. The other is asking questions directly in the notes tool, if it can search across all your meetings by person, company or project and cite the moment in the recording. For follow-ups and older decisions, the second is often enough and avoids moving transcripts around. Whichever you pick, make sure decisions and action items are stored as structured items rather than buried in summary prose, because that's what makes them retrievable months later.
 Lynkk is one built the second way, worth comparing with Fathom and Granola: on the paid plan you can ask across all your meetings by person, company or project, and every answer cites the moment in the recording.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Any Fathom AI alternatives that work better with agent workflows?</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Getting enough context from past meetings for follow-ups, tasks and older decisions means moving transcripts around by hand.</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/user/Sash19/</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/AI_Agents/comments/1wq1vrs/any_fathom_ai_alternatives_that_work_better_with/</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>"Fathom" alternative</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>comparison</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
@@ -1553,56 +1553,56 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/user/Nagib888/</t>
+          <t>post</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>post</t>
+          <t>https://www.reddit.com/r/MeetingsProductivity/comments/1xew8g2/do_meeting_templates_actually_help_or_do_they/</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/MeetingsProductivity/comments/1xew8g2/do_meeting_templates_actually_help_or_do_they/</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/MeetingsProductivity/comments/1xew8g2/do_meeting_templates_actually_help_or_do_they/</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Do meeting templates actually help, or do they create more work?</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>"action items" template</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>general_discussion</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr">
-        <is>
-          <t>Asks whether meeting templates help and which sections people reread.</t>
-        </is>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>Different templates per meeting type, but keep each short. The sections that hold up a week later are decisions, action items with owner and date, and open questions. Objectives and discussion notes rarely get reread. For a weekly check-in, blockers plus action items is enough; for discovery calls, the customer's problem in their own words plus next steps.
 What cuts the admin is letting the template fill itself from the recording. Lynkk, for example, has built-in formats for stand-ups, 1:1s, sales calls, customer interviews and product reviews (paid plan); Otter, Fireflies and Fathom are the other common ones to compare. It doesn't do custom formats, so if your sections are very specific a doc template still wins.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Do meeting templates actually help, or do they create more work?</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Asks whether meeting templates help and which sections people reread.</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/user/Nagib888/</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/MeetingsProductivity/comments/1xew8g2/do_meeting_templates_actually_help_or_do_they/</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>"action items" template</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>general_discussion</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
@@ -1644,56 +1644,56 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/user/kamikazekumako/</t>
+          <t>post</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>post</t>
+          <t>https://www.reddit.com/r/AI_Agents/comments/1wmwtl6/what_makes_a_good_ai_meeting_assistant/</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/AI_Agents/comments/1wmwtl6/what_makes_a_good_ai_meeting_assistant/</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/AI_Agents/comments/1wmwtl6/what_makes_a_good_ai_meeting_assistant/</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>What makes a good AI meeting assistant?</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>AI meeting assistant</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>tool_recommendation</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="inlineStr">
-        <is>
-          <t>Many in-person meetings daily; bots unwelcome under NDA; record-export-paste into ChatGPT is too many steps.</t>
-        </is>
-      </c>
-      <c r="N14" s="2" t="inlineStr">
         <is>
           <t>The step that kills it is the export and paste, so pick a tool where the recording and the organised notes live in one place. For NDA calls, a recorder on your own computer avoids the bot problem entirely. For in-person, a laptop in the middle of the table is usually enough for a few people.
 Lynkk is one to try next to Granola or Otter for that setup: it records in-person meetings from the browser, calls from a Mac app with no bot joining, and the brief pulls out decisions, action items and open questions automatically. It has no phone app though, so site visits without a laptop won't fit.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>What makes a good AI meeting assistant?</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Many in-person meetings daily; bots unwelcome under NDA; record-export-paste into ChatGPT is too many steps.</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/user/kamikazekumako/</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/AI_Agents/comments/1wmwtl6/what_makes_a_good_ai_meeting_assistant/</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>AI meeting assistant</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>tool_recommendation</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
@@ -1735,56 +1735,56 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/user/secondfillet/</t>
+          <t>post</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>post</t>
+          <t>https://www.reddit.com/r/Enterprise_AI_Agents/comments/1xcebs0/getting_an_ai_meeting_note_taker_for_microsoft/</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/Enterprise_AI_Agents/comments/1xcebs0/getting_an_ai_meeting_note_taker_for_microsoft/</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/Enterprise_AI_Agents/comments/1xcebs0/getting_an_ai_meeting_note_taker_for_microsoft/</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>Getting an AI meeting note taker for Microsoft Teams through security review</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>"note taker" sales</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="L15" s="2" t="inlineStr">
-        <is>
-          <t>tool_recommendation</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="inlineStr">
-        <is>
-          <t>Security review for a Teams note taker is a three-week document hunt: training, storage, subprocessors, retention.</t>
-        </is>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>The useful answers usually sit in three places: the DPA (retention, deletion, subprocessors), the trust or security page (certifications, storage location), and a written answer on model training. Get the training answer in writing, since it's the one that changes most often. A one-page table per vendor with exactly security's rows saves another round, and your feature comparison can wait.
 On the training row, Lynkk states it never trains on your conversations and keeps recordings private to each account. Otter, Fireflies and Copilot in Teams are the other names security teams usually line up. For certifications and storage location, ask each vendor directly rather than trusting the marketing page.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Getting an AI meeting note taker for Microsoft Teams through security review</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Security review for a Teams note taker is a three-week document hunt: training, storage, subprocessors, retention.</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/user/secondfillet/</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/Enterprise_AI_Agents/comments/1xcebs0/getting_an_ai_meeting_note_taker_for_microsoft/</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>"note taker" sales</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>tool_recommendation</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
@@ -1826,55 +1826,55 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
+          <t>comment</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/AgentsOfAI/comments/1xg9rj5/i_tested_6_ai_note_taking_tools_for_meetings/19rp9lez4ii5g/</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Same priorities here: no bot, and decisions and action items over a wall of text. If you want one more to test, Lynkk records without a bot from a Mac menu bar app or a Chrome extension and puts decisions and action items with owners in its brief. Granola and Otter are the other names that come up. Worth knowing the Mac app is Apple silicon only.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>I tested 6 AI note taking tools for meetings</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Needs no-bot capture and decisions/action items for long multi-person meetings.</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
           <t>https://www.reddit.com/user/Few_Importance_847/</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>comment</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/AgentsOfAI/comments/1xg9rj5/i_tested_6_ai_note_taking_tools_for_meetings/19rp9lez4ii5g/</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>https://www.reddit.com/r/AgentsOfAI/comments/1xg9rj5/i_tested_6_ai_note_taking_tools_for_meetings/</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>I tested 6 AI note taking tools for meetings</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>"meeting assistant" AI</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="K16" s="2" t="n">
+      <c r="M16" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>general_discussion</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="inlineStr">
-        <is>
-          <t>Needs no-bot capture and decisions/action items for long multi-person meetings.</t>
-        </is>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>Same priorities here: no bot, and decisions and action items over a wall of text. If you want one more to test, Lynkk records without a bot from a Mac menu bar app or a Chrome extension and puts decisions and action items with owners in its brief. Granola and Otter are the other names that come up. Worth knowing the Mac app is Apple silicon only.</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
@@ -1916,55 +1916,55 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
+          <t>post</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/Office365/comments/1x1dzwj/how_are_you_finding_ai_notetakers_connected_to/</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Turn off user consent for apps in Entra ID, or limit it to verified publishers with low-risk permissions, and switch on the admin consent workflow so requests come to you instead of running quietly. Then review Enterprise applications for anything holding Mail.Read or Calendars.Read, and alert on new consent grants. It also helps to approve one note taker centrally, otherwise people keep accepting whatever arrives in a meeting invite.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>How are you finding AI notetakers connected to your M365 tenant?</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>M365 admin found an AI note taker with mailbox read running quietly via user consent.</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
           <t>https://www.reddit.com/user/Henrieta_Awonusi/</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>post</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>https://www.reddit.com/r/Office365/comments/1x1dzwj/how_are_you_finding_ai_notetakers_connected_to/</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/Office365/comments/1x1dzwj/how_are_you_finding_ai_notetakers_connected_to/</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>How are you finding AI notetakers connected to your M365 tenant?</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>"note taker" sales</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="K17" s="2" t="n">
+      <c r="M17" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>general_discussion</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="inlineStr">
-        <is>
-          <t>M365 admin found an AI note taker with mailbox read running quietly via user consent.</t>
-        </is>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>Turn off user consent for apps in Entra ID, or limit it to verified publishers with low-risk permissions, and switch on the admin consent workflow so requests come to you instead of running quietly. Then review Enterprise applications for anything holding Mail.Read or Calendars.Read, and alert on new consent grants. It also helps to approve one note taker centrally, otherwise people keep accepting whatever arrives in a meeting invite.</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
@@ -2006,56 +2006,57 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
+          <t>post</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/Entrepreneurs/comments/1ws7c5b/other_alternative_for_business_when_everyone_has/</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>On migration: export each person's Otter history to files before switching and keep them in one shared place, rather than expecting the new tool to import them. Then move new meetings only, so nobody has to change habits overnight, and make offboarding part of the switch: one company account per person instead of personal sign-ups.
+Lynkk is worth a look next to Otter for Business and Fireflies for the management side: a company workspace where colleagues join by email domain, admins can read workspace notes (every admin read is logged), and people can still keep a note personal. It caps at 10 seats, so it suits small clients only.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Other alternative for business when everyone has a separate account?</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
           <t>https://www.reddit.com/user/Big-Personality-9618/</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>post</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>https://www.reddit.com/r/Entrepreneurs/comments/1ws7c5b/other_alternative_for_business_when_everyone_has/</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/Entrepreneurs/comments/1ws7c5b/other_alternative_for_business_when_everyone_has/</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>Other alternative for business when everyone has a separate account?</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>Otter alternative</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="K18" s="2" t="n">
+      <c r="M18" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>comparison</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr"/>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>(no reply: duplicate or weak fit, see reply_opportunity)</t>
-        </is>
-      </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
@@ -2092,55 +2093,55 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
+          <t>post</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/AiNoteTaker/comments/1xe7bui/not_a_notetaker_review_what_we_added_next_to_ours/</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Agree that a summary is written for the people who were on the call. One cheap thing that helps on handovers even without another tool: make the outgoing rep write a five-line "what's still true" note per account (open commitments, who decides, last objection, next date) and pin it in the CRM. Do you find the inheriting rep still checks the old calls, or does the account history replace that?</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Not a notetaker review: What we added next to ours and why</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Sales reps inheriting accounts lack prior call history; they layered an account-history tool over Gong.</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
           <t>https://www.reddit.com/user/Next_Classic_9664/</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>post</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>https://www.reddit.com/r/AiNoteTaker/comments/1xe7bui/not_a_notetaker_review_what_we_added_next_to_ours/</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/AiNoteTaker/comments/1xe7bui/not_a_notetaker_review_what_we_added_next_to_ours/</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>Not a notetaker review: What we added next to ours and why</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>"note taker" sales</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="K19" s="2" t="n">
+      <c r="M19" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>general_discussion</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="inlineStr">
-        <is>
-          <t>Sales reps inheriting accounts lack prior call history; they layered an account-history tool over Gong.</t>
-        </is>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>Agree that a summary is written for the people who were on the call. One cheap thing that helps on handovers even without another tool: make the outgoing rep write a five-line "what's still true" note per account (open commitments, who decides, last objection, next date) and pin it in the CRM. Do you find the inheriting rep still checks the old calls, or does the account history replace that?</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
@@ -2182,55 +2183,55 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
+          <t>post</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/MeetingsProductivity/comments/1vrrju0/best_tools_for_running_standups_that_dont_turn/</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Good list. One gap for live stand-ups: a recorder that pulls blockers and owners into a short note means nobody has to take minutes. Lynkk has a Daily Stand-up summary format for that (paid plan), and it pairs fine with Geekbot for the async days.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Best tools for running stand-ups that don’t turn into status theater (2026)</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Listicle on stand-up tools; nobody clear on owners after stand-ups.</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
           <t>https://www.reddit.com/user/TheAstrobro/</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>post</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr">
         <is>
           <t>https://www.reddit.com/r/MeetingsProductivity/comments/1vrrju0/best_tools_for_running_standups_that_dont_turn/</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/MeetingsProductivity/comments/1vrrju0/best_tools_for_running_standups_that_dont_turn/</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>Best tools for running stand-ups that don’t turn into status theater (2026)</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>"action items" template</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>2026-08-18</t>
         </is>
       </c>
-      <c r="K20" s="2" t="n">
+      <c r="M20" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="L20" s="2" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>general_discussion</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="inlineStr">
-        <is>
-          <t>Listicle on stand-up tools; nobody clear on owners after stand-ups.</t>
-        </is>
-      </c>
-      <c r="N20" s="2" t="inlineStr">
-        <is>
-          <t>Good list. One gap for live stand-ups: a recorder that pulls blockers and owners into a short note means nobody has to take minutes. Lynkk has a Daily Stand-up summary format for that (paid plan), and it pairs fine with Geekbot for the async days.</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
@@ -2272,60 +2273,61 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
+          <t>post</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/AiNoteTaker/comments/1vz63ez/any_deviceapp_that_does_it_all/</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>One tool that covers Teams, phone calls and face-to-face over a BT headset is rare, so it's often easier to split it: a desktop or browser recorder for Teams, a separate recorder for phone calls, and a laptop or recorder on the table for in-person meetings. Test the BT headset part carefully, since many headsets switch to a lower-quality mic mode during calls.
+For the Teams and face-to-face part, Lynkk is one to try alongside HiDock or Plaud: a Chrome extension records Teams in the browser on a PC without a bot, a meeting bot can join Teams links, and in-person meetings record from the browser. It doesn't record phone calls and has no iPhone app, so that part would still need something else.</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Any device/app that does it all?</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Wants one recorder for Teams, phone and in-person sales meetings.</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
           <t>https://www.reddit.com/user/Bigceps/</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>post</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="J21" s="2" t="inlineStr">
         <is>
           <t>https://www.reddit.com/r/AiNoteTaker/comments/1vz63ez/any_deviceapp_that_does_it_all/</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reddit.com/r/AiNoteTaker/comments/1vz63ez/any_deviceapp_that_does_it_all/</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>Any device/app that does it all?</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="K21" s="2" t="inlineStr">
         <is>
           <t>"note taker" sales</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="L21" s="2" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="K21" s="2" t="n">
+      <c r="M21" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="N21" s="2" t="inlineStr">
         <is>
           <t>tool_recommendation</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr">
-        <is>
-          <t>Wants one recorder for Teams, phone and in-person sales meetings.</t>
-        </is>
-      </c>
-      <c r="N21" s="2" t="inlineStr">
-        <is>
-          <t>(no reply: duplicate or weak fit, see reply_opportunity)</t>
-        </is>
-      </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">

</xml_diff>